<commit_message>
order files updated upto 22 oct 2026 Thursday
</commit_message>
<xml_diff>
--- a/ORDER_MGMT/regular_order_mgmt/order_files/FullOrders_upto_22oct26_Thurs.xlsx
+++ b/ORDER_MGMT/regular_order_mgmt/order_files/FullOrders_upto_22oct26_Thurs.xlsx
@@ -1898,7 +1898,7 @@
         <v>10880</v>
       </c>
       <c r="N2" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B2, $C$2:$C$620, C2, $D$2:$D$620, D2, $E$2:$E$620, E2) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" ref="N2:N65" si="0">IF(COUNTIFS( $B$2:$B$620, B2, $C$2:$C$620, C2, $D$2:$D$620, D2, $E$2:$E$620, E2) &gt; 1, "Duplicate", "Unique")</f>
         <v>Unique</v>
       </c>
       <c r="O2" s="10"/>
@@ -1946,7 +1946,7 @@
         <v>10680</v>
       </c>
       <c r="N3" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B3, $C$2:$C$620, C3, $D$2:$D$620, D3, $E$2:$E$620, E3) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O3" s="10"/>
@@ -1987,7 +1987,7 @@
       <c r="L4" s="16"/>
       <c r="M4" s="16"/>
       <c r="N4" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B4, $C$2:$C$620, C4, $D$2:$D$620, D4, $E$2:$E$620, E4) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2026,7 +2026,7 @@
       <c r="L5" s="16"/>
       <c r="M5" s="16"/>
       <c r="N5" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B5, $C$2:$C$620, C5, $D$2:$D$620, D5, $E$2:$E$620, E5) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2072,7 +2072,7 @@
         <v>450</v>
       </c>
       <c r="N6" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B6, $C$2:$C$620, C6, $D$2:$D$620, D6, $E$2:$E$620, E6) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O6" s="10"/>
@@ -2120,7 +2120,7 @@
         <v>1300</v>
       </c>
       <c r="N7" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B7, $C$2:$C$620, C7, $D$2:$D$620, D7, $E$2:$E$620, E7) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O7" s="10"/>
@@ -2168,7 +2168,7 @@
         <v>700</v>
       </c>
       <c r="N8" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B8, $C$2:$C$620, C8, $D$2:$D$620, D8, $E$2:$E$620, E8) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O8" s="10"/>
@@ -2207,7 +2207,7 @@
       <c r="L9" s="16"/>
       <c r="M9" s="16"/>
       <c r="N9" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B9, $C$2:$C$620, C9, $D$2:$D$620, D9, $E$2:$E$620, E9) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2253,7 +2253,7 @@
         <v>250</v>
       </c>
       <c r="N10" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B10, $C$2:$C$620, C10, $D$2:$D$620, D10, $E$2:$E$620, E10) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O10" s="10"/>
@@ -2301,7 +2301,7 @@
         <v>800</v>
       </c>
       <c r="N11" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B11, $C$2:$C$620, C11, $D$2:$D$620, D11, $E$2:$E$620, E11) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O11" s="10"/>
@@ -2340,7 +2340,7 @@
       <c r="L12" s="16"/>
       <c r="M12" s="16"/>
       <c r="N12" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B12, $C$2:$C$620, C12, $D$2:$D$620, D12, $E$2:$E$620, E12) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2386,7 +2386,7 @@
         <v>360</v>
       </c>
       <c r="N13" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B13, $C$2:$C$620, C13, $D$2:$D$620, D13, $E$2:$E$620, E13) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2426,7 +2426,7 @@
         <v>3156</v>
       </c>
       <c r="N14" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B14, $C$2:$C$620, C14, $D$2:$D$620, D14, $E$2:$E$620, E14) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="P14" s="18"/>
@@ -2473,7 +2473,7 @@
         <v>250</v>
       </c>
       <c r="N15" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B15, $C$2:$C$620, C15, $D$2:$D$620, D15, $E$2:$E$620, E15) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2512,7 +2512,7 @@
       <c r="L16" s="16"/>
       <c r="M16" s="16"/>
       <c r="N16" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B16, $C$2:$C$620, C16, $D$2:$D$620, D16, $E$2:$E$620, E16) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O16"/>
@@ -2560,7 +2560,7 @@
         <v>689.99999999999636</v>
       </c>
       <c r="N17" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B17, $C$2:$C$620, C17, $D$2:$D$620, D17, $E$2:$E$620, E17) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
         <v>225</v>
       </c>
       <c r="N18" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B18, $C$2:$C$620, C18, $D$2:$D$620, D18, $E$2:$E$620, E18) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O18" s="10"/>
@@ -2655,7 +2655,7 @@
         <v>660</v>
       </c>
       <c r="N19" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B19, $C$2:$C$620, C19, $D$2:$D$620, D19, $E$2:$E$620, E19) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2692,7 +2692,7 @@
       <c r="L20" s="16"/>
       <c r="M20" s="16"/>
       <c r="N20" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B20, $C$2:$C$620, C20, $D$2:$D$620, D20, $E$2:$E$620, E20) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O20"/>
@@ -2731,7 +2731,7 @@
       <c r="L21" s="16"/>
       <c r="M21" s="16"/>
       <c r="N21" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B21, $C$2:$C$620, C21, $D$2:$D$620, D21, $E$2:$E$620, E21) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O21"/>
@@ -2779,7 +2779,7 @@
         <v>250</v>
       </c>
       <c r="N22" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B22, $C$2:$C$620, C22, $D$2:$D$620, D22, $E$2:$E$620, E22) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -2825,7 +2825,7 @@
         <v>250</v>
       </c>
       <c r="N23" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B23, $C$2:$C$620, C23, $D$2:$D$620, D23, $E$2:$E$620, E23) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O23" s="10"/>
@@ -2864,7 +2864,7 @@
       <c r="L24" s="16"/>
       <c r="M24" s="16"/>
       <c r="N24" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B24, $C$2:$C$620, C24, $D$2:$D$620, D24, $E$2:$E$620, E24) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O24"/>
@@ -2905,7 +2905,7 @@
       <c r="L25" s="16"/>
       <c r="M25" s="16"/>
       <c r="N25" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B25, $C$2:$C$620, C25, $D$2:$D$620, D25, $E$2:$E$620, E25) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O25"/>
@@ -2954,7 +2954,7 @@
         <v>235</v>
       </c>
       <c r="N26" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B26, $C$2:$C$620, C26, $D$2:$D$620, D26, $E$2:$E$620, E26) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O26" s="10"/>
@@ -2993,7 +2993,7 @@
       <c r="L27" s="16"/>
       <c r="M27" s="16"/>
       <c r="N27" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B27, $C$2:$C$620, C27, $D$2:$D$620, D27, $E$2:$E$620, E27) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O27"/>
@@ -3032,7 +3032,7 @@
       <c r="L28" s="16"/>
       <c r="M28" s="16"/>
       <c r="N28" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B28, $C$2:$C$620, C28, $D$2:$D$620, D28, $E$2:$E$620, E28) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O28"/>
@@ -3076,11 +3076,11 @@
         <v>8239</v>
       </c>
       <c r="M29" s="17">
-        <f>ABS((D29*E29)-L29)</f>
+        <f t="shared" ref="M29:M34" si="1">ABS((D29*E29)-L29)</f>
         <v>528</v>
       </c>
       <c r="N29" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B29, $C$2:$C$620, C29, $D$2:$D$620, D29, $E$2:$E$620, E29) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O29" s="10"/>
@@ -3124,11 +3124,11 @@
         <v>34800</v>
       </c>
       <c r="M30" s="17">
-        <f>ABS((D30*E30)-L30)</f>
+        <f t="shared" si="1"/>
         <v>1600</v>
       </c>
       <c r="N30" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B30, $C$2:$C$620, C30, $D$2:$D$620, D30, $E$2:$E$620, E30) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Duplicate</v>
       </c>
       <c r="O30" s="10"/>
@@ -3172,11 +3172,11 @@
         <v>34400</v>
       </c>
       <c r="M31" s="17">
-        <f>ABS((D31*E31)-L31)</f>
+        <f t="shared" si="1"/>
         <v>1200</v>
       </c>
       <c r="N31" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B31, $C$2:$C$620, C31, $D$2:$D$620, D31, $E$2:$E$620, E31) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Duplicate</v>
       </c>
       <c r="O31" s="10"/>
@@ -3220,11 +3220,11 @@
         <v>33900</v>
       </c>
       <c r="M32" s="17">
-        <f>ABS((D32*E32)-L32)</f>
+        <f t="shared" si="1"/>
         <v>700</v>
       </c>
       <c r="N32" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B32, $C$2:$C$620, C32, $D$2:$D$620, D32, $E$2:$E$620, E32) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Duplicate</v>
       </c>
       <c r="O32" s="10"/>
@@ -3268,11 +3268,11 @@
         <v>33900</v>
       </c>
       <c r="M33" s="17">
-        <f>ABS((D33*E33)-L33)</f>
+        <f t="shared" si="1"/>
         <v>700</v>
       </c>
       <c r="N33" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B33, $C$2:$C$620, C33, $D$2:$D$620, D33, $E$2:$E$620, E33) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Duplicate</v>
       </c>
     </row>
@@ -3314,11 +3314,11 @@
         <v>33900</v>
       </c>
       <c r="M34" s="17">
-        <f>ABS((D34*E34)-L34)</f>
+        <f t="shared" si="1"/>
         <v>700</v>
       </c>
       <c r="N34" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B34, $C$2:$C$620, C34, $D$2:$D$620, D34, $E$2:$E$620, E34) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Duplicate</v>
       </c>
     </row>
@@ -3355,7 +3355,7 @@
       <c r="L35" s="16"/>
       <c r="M35" s="16"/>
       <c r="N35" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B35, $C$2:$C$620, C35, $D$2:$D$620, D35, $E$2:$E$620, E35) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O35"/>
@@ -3403,7 +3403,7 @@
         <v>250</v>
       </c>
       <c r="N36" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B36, $C$2:$C$620, C36, $D$2:$D$620, D36, $E$2:$E$620, E36) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3442,7 +3442,7 @@
       <c r="L37" s="16"/>
       <c r="M37" s="16"/>
       <c r="N37" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B37, $C$2:$C$620, C37, $D$2:$D$620, D37, $E$2:$E$620, E37) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O37"/>
@@ -3481,7 +3481,7 @@
       <c r="L38" s="16"/>
       <c r="M38" s="16"/>
       <c r="N38" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B38, $C$2:$C$620, C38, $D$2:$D$620, D38, $E$2:$E$620, E38) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O38"/>
@@ -3529,7 +3529,7 @@
         <v>300</v>
       </c>
       <c r="N39" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B39, $C$2:$C$620, C39, $D$2:$D$620, D39, $E$2:$E$620, E39) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3576,7 +3576,7 @@
         <v>448</v>
       </c>
       <c r="N40" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B40, $C$2:$C$620, C40, $D$2:$D$620, D40, $E$2:$E$620, E40) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3623,7 +3623,7 @@
         <v>135</v>
       </c>
       <c r="N41" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B41, $C$2:$C$620, C41, $D$2:$D$620, D41, $E$2:$E$620, E41) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3660,7 +3660,7 @@
       <c r="L42" s="16"/>
       <c r="M42" s="16"/>
       <c r="N42" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B42, $C$2:$C$620, C42, $D$2:$D$620, D42, $E$2:$E$620, E42) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O42"/>
@@ -3701,7 +3701,7 @@
       <c r="L43" s="16"/>
       <c r="M43" s="16"/>
       <c r="N43" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B43, $C$2:$C$620, C43, $D$2:$D$620, D43, $E$2:$E$620, E43) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O43"/>
@@ -3749,7 +3749,7 @@
         <v>650</v>
       </c>
       <c r="N44" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B44, $C$2:$C$620, C44, $D$2:$D$620, D44, $E$2:$E$620, E44) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3795,7 +3795,7 @@
         <v>295</v>
       </c>
       <c r="N45" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B45, $C$2:$C$620, C45, $D$2:$D$620, D45, $E$2:$E$620, E45) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O45" s="10"/>
@@ -3834,7 +3834,7 @@
       <c r="L46" s="16"/>
       <c r="M46" s="16"/>
       <c r="N46" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B46, $C$2:$C$620, C46, $D$2:$D$620, D46, $E$2:$E$620, E46) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O46"/>
@@ -3882,7 +3882,7 @@
         <v>253</v>
       </c>
       <c r="N47" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B47, $C$2:$C$620, C47, $D$2:$D$620, D47, $E$2:$E$620, E47) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -3919,7 +3919,7 @@
       <c r="L48" s="16"/>
       <c r="M48" s="16"/>
       <c r="N48" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B48, $C$2:$C$620, C48, $D$2:$D$620, D48, $E$2:$E$620, E48) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O48"/>
@@ -3968,7 +3968,7 @@
         <v>540</v>
       </c>
       <c r="N49" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B49, $C$2:$C$620, C49, $D$2:$D$620, D49, $E$2:$E$620, E49) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O49"/>
@@ -4016,7 +4016,7 @@
         <v>300</v>
       </c>
       <c r="N50" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B50, $C$2:$C$620, C50, $D$2:$D$620, D50, $E$2:$E$620, E50) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4053,7 +4053,7 @@
       <c r="L51" s="16"/>
       <c r="M51" s="16"/>
       <c r="N51" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B51, $C$2:$C$620, C51, $D$2:$D$620, D51, $E$2:$E$620, E51) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O51"/>
@@ -4101,7 +4101,7 @@
         <v>264</v>
       </c>
       <c r="N52" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B52, $C$2:$C$620, C52, $D$2:$D$620, D52, $E$2:$E$620, E52) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4148,7 +4148,7 @@
         <v>220</v>
       </c>
       <c r="N53" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B53, $C$2:$C$620, C53, $D$2:$D$620, D53, $E$2:$E$620, E53) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4194,7 +4194,7 @@
         <v>240</v>
       </c>
       <c r="N54" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B54, $C$2:$C$620, C54, $D$2:$D$620, D54, $E$2:$E$620, E54) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4233,7 +4233,7 @@
       <c r="L55" s="16"/>
       <c r="M55" s="16"/>
       <c r="N55" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B55, $C$2:$C$620, C55, $D$2:$D$620, D55, $E$2:$E$620, E55) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4267,7 +4267,7 @@
       </c>
       <c r="J56" s="32"/>
       <c r="N56" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B56, $C$2:$C$620, C56, $D$2:$D$620, D56, $E$2:$E$620, E56) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O56" s="27"/>
@@ -4314,7 +4314,7 @@
         <v>2300</v>
       </c>
       <c r="N57" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B57, $C$2:$C$620, C57, $D$2:$D$620, D57, $E$2:$E$620, E57) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O57" s="27"/>
@@ -4352,7 +4352,7 @@
       <c r="L58" s="16"/>
       <c r="M58" s="16"/>
       <c r="N58" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B58, $C$2:$C$620, C58, $D$2:$D$620, D58, $E$2:$E$620, E58) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O58"/>
@@ -4394,7 +4394,7 @@
       <c r="L59" s="16"/>
       <c r="M59" s="16"/>
       <c r="N59" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B59, $C$2:$C$620, C59, $D$2:$D$620, D59, $E$2:$E$620, E59) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O59"/>
@@ -4443,7 +4443,7 @@
         <v>440</v>
       </c>
       <c r="N60" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B60, $C$2:$C$620, C60, $D$2:$D$620, D60, $E$2:$E$620, E60) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4482,7 +4482,7 @@
       <c r="L61" s="61"/>
       <c r="M61" s="61"/>
       <c r="N61" s="62" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B61, $C$2:$C$620, C61, $D$2:$D$620, D61, $E$2:$E$620, E61) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O61" s="63"/>
@@ -4518,7 +4518,7 @@
       </c>
       <c r="J62" s="32"/>
       <c r="N62" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B62, $C$2:$C$620, C62, $D$2:$D$620, D62, $E$2:$E$620, E62) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4557,7 +4557,7 @@
       <c r="L63" s="16"/>
       <c r="M63" s="16"/>
       <c r="N63" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B63, $C$2:$C$620, C63, $D$2:$D$620, D63, $E$2:$E$620, E63) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O63"/>
@@ -4605,7 +4605,7 @@
         <v>300</v>
       </c>
       <c r="N64" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B64, $C$2:$C$620, C64, $D$2:$D$620, D64, $E$2:$E$620, E64) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4644,7 +4644,7 @@
       <c r="L65" s="16"/>
       <c r="M65" s="16"/>
       <c r="N65" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B65, $C$2:$C$620, C65, $D$2:$D$620, D65, $E$2:$E$620, E65) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
       <c r="O65"/>
@@ -4692,7 +4692,7 @@
         <v>470</v>
       </c>
       <c r="N66" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B66, $C$2:$C$620, C66, $D$2:$D$620, D66, $E$2:$E$620, E66) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" ref="N66:N129" si="2">IF(COUNTIFS( $B$2:$B$620, B66, $C$2:$C$620, C66, $D$2:$D$620, D66, $E$2:$E$620, E66) &gt; 1, "Duplicate", "Unique")</f>
         <v>Unique</v>
       </c>
     </row>
@@ -4731,7 +4731,7 @@
       <c r="L67" s="62"/>
       <c r="M67" s="61"/>
       <c r="N67" s="63" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B67, $C$2:$C$620, C67, $D$2:$D$620, D67, $E$2:$E$620, E67) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
       <c r="O67" s="63"/>
@@ -4772,7 +4772,7 @@
       <c r="L68" s="17"/>
       <c r="M68" s="17"/>
       <c r="N68" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B68, $C$2:$C$620, C68, $D$2:$D$620, D68, $E$2:$E$620, E68) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
       <c r="O68" s="10"/>
@@ -4820,7 +4820,7 @@
         <v>700</v>
       </c>
       <c r="N69" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B69, $C$2:$C$620, C69, $D$2:$D$620, D69, $E$2:$E$620, E69) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4859,7 +4859,7 @@
       <c r="L70" s="16"/>
       <c r="M70" s="16"/>
       <c r="N70" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B70, $C$2:$C$620, C70, $D$2:$D$620, D70, $E$2:$E$620, E70) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
       <c r="O70"/>
@@ -4908,7 +4908,7 @@
         <v>240</v>
       </c>
       <c r="N71" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B71, $C$2:$C$620, C71, $D$2:$D$620, D71, $E$2:$E$620, E71) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -4947,7 +4947,7 @@
       <c r="L72" s="16"/>
       <c r="M72" s="16"/>
       <c r="N72" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B72, $C$2:$C$620, C72, $D$2:$D$620, D72, $E$2:$E$620, E72) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
       <c r="O72" s="10"/>
@@ -4988,7 +4988,7 @@
       <c r="L73" s="16"/>
       <c r="M73" s="16"/>
       <c r="N73" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B73, $C$2:$C$620, C73, $D$2:$D$620, D73, $E$2:$E$620, E73) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
       <c r="P73"/>
@@ -5035,7 +5035,7 @@
         <v>295</v>
       </c>
       <c r="N74" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B74, $C$2:$C$620, C74, $D$2:$D$620, D74, $E$2:$E$620, E74) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5074,7 +5074,7 @@
       <c r="L75" s="61"/>
       <c r="M75" s="61"/>
       <c r="N75" s="62" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B75, $C$2:$C$620, C75, $D$2:$D$620, D75, $E$2:$E$620, E75) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
       <c r="O75" s="63"/>
@@ -5113,7 +5113,7 @@
       <c r="L76" s="16"/>
       <c r="M76" s="16"/>
       <c r="N76" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B76, $C$2:$C$620, C76, $D$2:$D$620, D76, $E$2:$E$620, E76) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
       <c r="O76"/>
@@ -5161,7 +5161,7 @@
         <v>720</v>
       </c>
       <c r="N77" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B77, $C$2:$C$620, C77, $D$2:$D$620, D77, $E$2:$E$620, E77) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5198,7 +5198,7 @@
       <c r="L78" s="16"/>
       <c r="M78" s="16"/>
       <c r="N78" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B78, $C$2:$C$620, C78, $D$2:$D$620, D78, $E$2:$E$620, E78) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5244,7 +5244,7 @@
         <v>840</v>
       </c>
       <c r="N79" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B79, $C$2:$C$620, C79, $D$2:$D$620, D79, $E$2:$E$620, E79) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5281,7 +5281,7 @@
       <c r="L80" s="16"/>
       <c r="M80" s="16"/>
       <c r="N80" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B80, $C$2:$C$620, C80, $D$2:$D$620, D80, $E$2:$E$620, E80) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5320,7 +5320,7 @@
       <c r="L81" s="61"/>
       <c r="M81" s="61"/>
       <c r="N81" s="62" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B81, $C$2:$C$620, C81, $D$2:$D$620, D81, $E$2:$E$620, E81) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
       <c r="O81" s="63"/>
@@ -5368,7 +5368,7 @@
         <v>660</v>
       </c>
       <c r="N82" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B82, $C$2:$C$620, C82, $D$2:$D$620, D82, $E$2:$E$620, E82) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
       <c r="O82" s="10"/>
@@ -5416,7 +5416,7 @@
         <v>700</v>
       </c>
       <c r="N83" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B83, $C$2:$C$620, C83, $D$2:$D$620, D83, $E$2:$E$620, E83) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
       <c r="O83" s="10"/>
@@ -5452,7 +5452,7 @@
       </c>
       <c r="J84" s="32"/>
       <c r="N84" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B84, $C$2:$C$620, C84, $D$2:$D$620, D84, $E$2:$E$620, E84) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5488,7 +5488,7 @@
         <v>117</v>
       </c>
       <c r="N85" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B85, $C$2:$C$620, C85, $D$2:$D$620, D85, $E$2:$E$620, E85) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
       <c r="O85" s="27"/>
@@ -5526,7 +5526,7 @@
       <c r="L86" s="16"/>
       <c r="M86" s="16"/>
       <c r="N86" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B86, $C$2:$C$620, C86, $D$2:$D$620, D86, $E$2:$E$620, E86) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
       <c r="O86" s="18"/>
@@ -5574,7 +5574,7 @@
         <v>920</v>
       </c>
       <c r="N87" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B87, $C$2:$C$620, C87, $D$2:$D$620, D87, $E$2:$E$620, E87) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5613,7 +5613,7 @@
       <c r="L88" s="16"/>
       <c r="M88" s="16"/>
       <c r="N88" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B88, $C$2:$C$620, C88, $D$2:$D$620, D88, $E$2:$E$620, E88) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
       <c r="O88"/>
@@ -5661,7 +5661,7 @@
         <v>300</v>
       </c>
       <c r="N89" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B89, $C$2:$C$620, C89, $D$2:$D$620, D89, $E$2:$E$620, E89) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
       <c r="P89" s="22"/>
@@ -5709,7 +5709,7 @@
         <v>260</v>
       </c>
       <c r="N90" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B90, $C$2:$C$620, C90, $D$2:$D$620, D90, $E$2:$E$620, E90) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5755,7 +5755,7 @@
         <v>516</v>
       </c>
       <c r="N91" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B91, $C$2:$C$620, C91, $D$2:$D$620, D91, $E$2:$E$620, E91) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5794,7 +5794,7 @@
       <c r="L92" s="17"/>
       <c r="M92" s="17"/>
       <c r="N92" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B92, $C$2:$C$620, C92, $D$2:$D$620, D92, $E$2:$E$620, E92) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
       <c r="O92" s="10"/>
@@ -5842,7 +5842,7 @@
         <v>393</v>
       </c>
       <c r="N93" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B93, $C$2:$C$620, C93, $D$2:$D$620, D93, $E$2:$E$620, E93) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
       <c r="O93" s="10"/>
@@ -5890,7 +5890,7 @@
         <v>660</v>
       </c>
       <c r="N94" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B94, $C$2:$C$620, C94, $D$2:$D$620, D94, $E$2:$E$620, E94) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -5927,7 +5927,7 @@
       <c r="L95" s="16"/>
       <c r="M95" s="16"/>
       <c r="N95" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B95, $C$2:$C$620, C95, $D$2:$D$620, D95, $E$2:$E$620, E95) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
       <c r="O95" s="23"/>
@@ -5970,11 +5970,11 @@
         <v>14560</v>
       </c>
       <c r="M96" s="17">
-        <f>ABS((D96*E96)-L96)</f>
+        <f t="shared" ref="M96:M102" si="3">ABS((D96*E96)-L96)</f>
         <v>300</v>
       </c>
       <c r="N96" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B96, $C$2:$C$620, C96, $D$2:$D$620, D96, $E$2:$E$620, E96) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6017,11 +6017,11 @@
         <v>8870</v>
       </c>
       <c r="M97" s="17">
-        <f>ABS((D97*E97)-L97)</f>
+        <f t="shared" si="3"/>
         <v>200</v>
       </c>
       <c r="N97" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B97, $C$2:$C$620, C97, $D$2:$D$620, D97, $E$2:$E$620, E97) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6063,11 +6063,11 @@
         <v>8220</v>
       </c>
       <c r="M98" s="17">
-        <f>ABS((D98*E98)-L98)</f>
+        <f t="shared" si="3"/>
         <v>360</v>
       </c>
       <c r="N98" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B98, $C$2:$C$620, C98, $D$2:$D$620, D98, $E$2:$E$620, E98) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
       <c r="O98" s="35" t="s">
@@ -6112,11 +6112,11 @@
         <v>15075</v>
       </c>
       <c r="M99" s="17">
-        <f>ABS((D99*E99)-L99)</f>
+        <f t="shared" si="3"/>
         <v>645</v>
       </c>
       <c r="N99" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B99, $C$2:$C$620, C99, $D$2:$D$620, D99, $E$2:$E$620, E99) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
       <c r="O99" s="35" t="s">
@@ -6161,11 +6161,11 @@
         <v>17020</v>
       </c>
       <c r="M100" s="17">
-        <f>ABS((D100*E100)-L100)</f>
+        <f t="shared" si="3"/>
         <v>650</v>
       </c>
       <c r="N100" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B100, $C$2:$C$620, C100, $D$2:$D$620, D100, $E$2:$E$620, E100) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6207,11 +6207,11 @@
         <v>6756</v>
       </c>
       <c r="M101" s="17">
-        <f>ABS((D101*E101)-L101)</f>
+        <f t="shared" si="3"/>
         <v>390</v>
       </c>
       <c r="N101" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B101, $C$2:$C$620, C101, $D$2:$D$620, D101, $E$2:$E$620, E101) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6253,11 +6253,11 @@
         <v>2979</v>
       </c>
       <c r="M102" s="17">
-        <f>ABS((D102*E102)-L102)</f>
+        <f t="shared" si="3"/>
         <v>250</v>
       </c>
       <c r="N102" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B102, $C$2:$C$620, C102, $D$2:$D$620, D102, $E$2:$E$620, E102) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6291,7 +6291,7 @@
       </c>
       <c r="J103" s="32"/>
       <c r="N103" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B103, $C$2:$C$620, C103, $D$2:$D$620, D103, $E$2:$E$620, E103) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6330,7 +6330,7 @@
       <c r="L104" s="16"/>
       <c r="M104" s="16"/>
       <c r="N104" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B104, $C$2:$C$620, C104, $D$2:$D$620, D104, $E$2:$E$620, E104) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
       <c r="O104"/>
@@ -6374,11 +6374,11 @@
         <v>14310</v>
       </c>
       <c r="M105" s="17">
-        <f>ABS((D105*E105)-L105)</f>
+        <f t="shared" ref="M105:M112" si="4">ABS((D105*E105)-L105)</f>
         <v>660</v>
       </c>
       <c r="N105" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B105, $C$2:$C$620, C105, $D$2:$D$620, D105, $E$2:$E$620, E105) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6421,11 +6421,11 @@
         <v>8870</v>
       </c>
       <c r="M106" s="17">
-        <f>ABS((D106*E106)-L106)</f>
+        <f t="shared" si="4"/>
         <v>300</v>
       </c>
       <c r="N106" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B106, $C$2:$C$620, C106, $D$2:$D$620, D106, $E$2:$E$620, E106) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
       <c r="O106" s="35" t="s">
@@ -6470,11 +6470,11 @@
         <v>10300</v>
       </c>
       <c r="M107" s="17">
-        <f>ABS((D107*E107)-L107)</f>
+        <f t="shared" si="4"/>
         <v>300</v>
       </c>
       <c r="N107" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B107, $C$2:$C$620, C107, $D$2:$D$620, D107, $E$2:$E$620, E107) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
       <c r="P107" s="27"/>
@@ -6517,11 +6517,11 @@
         <v>11694</v>
       </c>
       <c r="M108" s="17">
-        <f>ABS((D108*E108)-L108)</f>
+        <f t="shared" si="4"/>
         <v>1000</v>
       </c>
       <c r="N108" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B108, $C$2:$C$620, C108, $D$2:$D$620, D108, $E$2:$E$620, E108) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
       <c r="O108" s="10"/>
@@ -6565,11 +6565,11 @@
         <v>8422.5</v>
       </c>
       <c r="M109" s="17">
-        <f>ABS((D109*E109)-L109)</f>
+        <f t="shared" si="4"/>
         <v>277.5</v>
       </c>
       <c r="N109" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B109, $C$2:$C$620, C109, $D$2:$D$620, D109, $E$2:$E$620, E109) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6611,11 +6611,11 @@
         <v>2593</v>
       </c>
       <c r="M110" s="17">
-        <f>ABS((D110*E110)-L110)</f>
+        <f t="shared" si="4"/>
         <v>250</v>
       </c>
       <c r="N110" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B110, $C$2:$C$620, C110, $D$2:$D$620, D110, $E$2:$E$620, E110) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6657,11 +6657,11 @@
         <v>17310</v>
       </c>
       <c r="M111" s="17">
-        <f>ABS((D111*E111)-L111)</f>
+        <f t="shared" si="4"/>
         <v>650</v>
       </c>
       <c r="N111" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B111, $C$2:$C$620, C111, $D$2:$D$620, D111, $E$2:$E$620, E111) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6703,11 +6703,11 @@
         <v>8420</v>
       </c>
       <c r="M112" s="17">
-        <f>ABS((D112*E112)-L112)</f>
+        <f t="shared" si="4"/>
         <v>300</v>
       </c>
       <c r="N112" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B112, $C$2:$C$620, C112, $D$2:$D$620, D112, $E$2:$E$620, E112) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6746,7 +6746,7 @@
       <c r="L113" s="16"/>
       <c r="M113" s="16"/>
       <c r="N113" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B113, $C$2:$C$620, C113, $D$2:$D$620, D113, $E$2:$E$620, E113) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6788,11 +6788,11 @@
         <v>6127.5</v>
       </c>
       <c r="M114" s="25">
-        <f>ABS((D114*E114)-L114)</f>
+        <f t="shared" ref="M114:M122" si="5">ABS((D114*E114)-L114)</f>
         <v>612.5</v>
       </c>
       <c r="N114" s="27" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B114, $C$2:$C$620, C114, $D$2:$D$620, D114, $E$2:$E$620, E114) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Duplicate</v>
       </c>
       <c r="O114" s="27"/>
@@ -6836,11 +6836,11 @@
         <v>6320</v>
       </c>
       <c r="M115" s="25">
-        <f>ABS((D115*E115)-L115)</f>
+        <f t="shared" si="5"/>
         <v>420</v>
       </c>
       <c r="N115" s="27" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B115, $C$2:$C$620, C115, $D$2:$D$620, D115, $E$2:$E$620, E115) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Duplicate</v>
       </c>
       <c r="O115" s="27"/>
@@ -6885,11 +6885,11 @@
         <v>8970</v>
       </c>
       <c r="M116" s="17">
-        <f>ABS((D116*E116)-L116)</f>
+        <f t="shared" si="5"/>
         <v>300</v>
       </c>
       <c r="N116" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B116, $C$2:$C$620, C116, $D$2:$D$620, D116, $E$2:$E$620, E116) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -6931,11 +6931,11 @@
         <v>10410</v>
       </c>
       <c r="M117" s="17">
-        <f>ABS((D117*E117)-L117)</f>
+        <f t="shared" si="5"/>
         <v>300</v>
       </c>
       <c r="N117" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B117, $C$2:$C$620, C117, $D$2:$D$620, D117, $E$2:$E$620, E117) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
       <c r="O117" s="27"/>
@@ -6978,11 +6978,11 @@
         <v>6868</v>
       </c>
       <c r="M118" s="17">
-        <f>ABS((D118*E118)-L118)</f>
+        <f t="shared" si="5"/>
         <v>300</v>
       </c>
       <c r="N118" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B118, $C$2:$C$620, C118, $D$2:$D$620, D118, $E$2:$E$620, E118) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7024,11 +7024,11 @@
         <v>4036</v>
       </c>
       <c r="M119" s="17">
-        <f>ABS((D119*E119)-L119)</f>
+        <f t="shared" si="5"/>
         <v>404</v>
       </c>
       <c r="N119" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B119, $C$2:$C$620, C119, $D$2:$D$620, D119, $E$2:$E$620, E119) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7070,11 +7070,11 @@
         <v>9170</v>
       </c>
       <c r="M120" s="25">
-        <f>ABS((D120*E120)-L120)</f>
+        <f t="shared" si="5"/>
         <v>200</v>
       </c>
       <c r="N120" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B120, $C$2:$C$620, C120, $D$2:$D$620, D120, $E$2:$E$620, E120) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7116,11 +7116,11 @@
         <v>19730.5</v>
       </c>
       <c r="M121" s="25">
-        <f>ABS((D121*E121)-L121)</f>
+        <f t="shared" si="5"/>
         <v>504.5</v>
       </c>
       <c r="N121" s="27" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B121, $C$2:$C$620, C121, $D$2:$D$620, D121, $E$2:$E$620, E121) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Duplicate</v>
       </c>
       <c r="O121" s="35" t="s">
@@ -7166,11 +7166,11 @@
         <v>19690</v>
       </c>
       <c r="M122" s="25">
-        <f>ABS((D122*E122)-L122)</f>
+        <f t="shared" si="5"/>
         <v>545</v>
       </c>
       <c r="N122" s="27" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B122, $C$2:$C$620, C122, $D$2:$D$620, D122, $E$2:$E$620, E122) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Duplicate</v>
       </c>
       <c r="O122" s="35" t="s">
@@ -7208,7 +7208,7 @@
       </c>
       <c r="J123" s="32"/>
       <c r="N123" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B123, $C$2:$C$620, C123, $D$2:$D$620, D123, $E$2:$E$620, E123) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7255,7 +7255,7 @@
         <v>444</v>
       </c>
       <c r="N124" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B124, $C$2:$C$620, C124, $D$2:$D$620, D124, $E$2:$E$620, E124) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7301,7 +7301,7 @@
         <v>300</v>
       </c>
       <c r="N125" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B125, $C$2:$C$620, C125, $D$2:$D$620, D125, $E$2:$E$620, E125) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7340,7 +7340,7 @@
       <c r="L126" s="16"/>
       <c r="M126" s="16"/>
       <c r="N126" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B126, $C$2:$C$620, C126, $D$2:$D$620, D126, $E$2:$E$620, E126) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7382,11 +7382,11 @@
         <v>9886</v>
       </c>
       <c r="M127" s="17">
-        <f>ABS((D127*E127)-L127)</f>
+        <f t="shared" ref="M127:M139" si="6">ABS((D127*E127)-L127)</f>
         <v>654</v>
       </c>
       <c r="N127" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B127, $C$2:$C$620, C127, $D$2:$D$620, D127, $E$2:$E$620, E127) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
       <c r="O127" s="35" t="s">
@@ -7432,11 +7432,11 @@
         <v>17040</v>
       </c>
       <c r="M128" s="17">
-        <f>ABS((D128*E128)-L128)</f>
+        <f t="shared" si="6"/>
         <v>880</v>
       </c>
       <c r="N128" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B128, $C$2:$C$620, C128, $D$2:$D$620, D128, $E$2:$E$620, E128) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
       <c r="O128" s="35" t="s">
@@ -7481,11 +7481,11 @@
         <v>18495</v>
       </c>
       <c r="M129" s="17">
-        <f>ABS((D129*E129)-L129)</f>
+        <f t="shared" si="6"/>
         <v>900</v>
       </c>
       <c r="N129" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B129, $C$2:$C$620, C129, $D$2:$D$620, D129, $E$2:$E$620, E129) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7527,11 +7527,11 @@
         <v>39300</v>
       </c>
       <c r="M130" s="17">
-        <f>ABS((D130*E130)-L130)</f>
+        <f t="shared" si="6"/>
         <v>18850</v>
       </c>
       <c r="N130" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B130, $C$2:$C$620, C130, $D$2:$D$620, D130, $E$2:$E$620, E130) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" ref="N130:N193" si="7">IF(COUNTIFS( $B$2:$B$620, B130, $C$2:$C$620, C130, $D$2:$D$620, D130, $E$2:$E$620, E130) &gt; 1, "Duplicate", "Unique")</f>
         <v>Unique</v>
       </c>
     </row>
@@ -7573,11 +7573,11 @@
         <v>9170</v>
       </c>
       <c r="M131" s="25">
-        <f>ABS((D131*E131)-L131)</f>
+        <f t="shared" si="6"/>
         <v>300</v>
       </c>
       <c r="N131" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B131, $C$2:$C$620, C131, $D$2:$D$620, D131, $E$2:$E$620, E131) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7619,11 +7619,11 @@
         <v>20010</v>
       </c>
       <c r="M132" s="17">
-        <f>ABS((D132*E132)-L132)</f>
+        <f t="shared" si="6"/>
         <v>450</v>
       </c>
       <c r="N132" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B132, $C$2:$C$620, C132, $D$2:$D$620, D132, $E$2:$E$620, E132) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
       <c r="P132"/>
@@ -7666,11 +7666,11 @@
         <v>8570</v>
       </c>
       <c r="M133" s="25">
-        <f>ABS((D133*E133)-L133)</f>
+        <f t="shared" si="6"/>
         <v>650</v>
       </c>
       <c r="N133" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B133, $C$2:$C$620, C133, $D$2:$D$620, D133, $E$2:$E$620, E133) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
       <c r="O133" s="35" t="s">
@@ -7715,11 +7715,11 @@
         <v>21900</v>
       </c>
       <c r="M134" s="17">
-        <f>ABS((D134*E134)-L134)</f>
+        <f t="shared" si="6"/>
         <v>500</v>
       </c>
       <c r="N134" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B134, $C$2:$C$620, C134, $D$2:$D$620, D134, $E$2:$E$620, E134) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7761,11 +7761,11 @@
         <v>4852</v>
       </c>
       <c r="M135" s="17">
-        <f>ABS((D135*E135)-L135)</f>
+        <f t="shared" si="6"/>
         <v>274</v>
       </c>
       <c r="N135" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B135, $C$2:$C$620, C135, $D$2:$D$620, D135, $E$2:$E$620, E135) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
       <c r="O135" s="10"/>
@@ -7809,11 +7809,11 @@
         <v>8700</v>
       </c>
       <c r="M136" s="17">
-        <f>ABS((D136*E136)-L136)</f>
+        <f t="shared" si="6"/>
         <v>250</v>
       </c>
       <c r="N136" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B136, $C$2:$C$620, C136, $D$2:$D$620, D136, $E$2:$E$620, E136) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7855,11 +7855,11 @@
         <v>20260</v>
       </c>
       <c r="M137" s="17">
-        <f>ABS((D137*E137)-L137)</f>
+        <f t="shared" si="6"/>
         <v>300</v>
       </c>
       <c r="N137" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B137, $C$2:$C$620, C137, $D$2:$D$620, D137, $E$2:$E$620, E137) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
       <c r="O137"/>
@@ -7903,11 +7903,11 @@
         <v>13237.5</v>
       </c>
       <c r="M138" s="17">
-        <f>ABS((D138*E138)-L138)</f>
+        <f t="shared" si="6"/>
         <v>1000</v>
       </c>
       <c r="N138" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B138, $C$2:$C$620, C138, $D$2:$D$620, D138, $E$2:$E$620, E138) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -7949,11 +7949,11 @@
         <v>5620</v>
       </c>
       <c r="M139" s="25">
-        <f>ABS((D139*E139)-L139)</f>
+        <f t="shared" si="6"/>
         <v>300</v>
       </c>
       <c r="N139" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B139, $C$2:$C$620, C139, $D$2:$D$620, D139, $E$2:$E$620, E139) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
       <c r="P139" s="23"/>
@@ -7988,7 +7988,7 @@
       </c>
       <c r="J140" s="32"/>
       <c r="N140" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B140, $C$2:$C$620, C140, $D$2:$D$620, D140, $E$2:$E$620, E140) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -8034,7 +8034,7 @@
         <v>300</v>
       </c>
       <c r="N141" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B141, $C$2:$C$620, C141, $D$2:$D$620, D141, $E$2:$E$620, E141) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
       <c r="P141" s="18"/>
@@ -8071,7 +8071,7 @@
         <v>117</v>
       </c>
       <c r="N142" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B142, $C$2:$C$620, C142, $D$2:$D$620, D142, $E$2:$E$620, E142) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -8117,7 +8117,7 @@
         <v>1028.25</v>
       </c>
       <c r="N143" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B143, $C$2:$C$620, C143, $D$2:$D$620, D143, $E$2:$E$620, E143) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -8153,7 +8153,7 @@
         <v>116</v>
       </c>
       <c r="N144" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B144, $C$2:$C$620, C144, $D$2:$D$620, D144, $E$2:$E$620, E144) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -8187,7 +8187,7 @@
       </c>
       <c r="J145" s="32"/>
       <c r="N145" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B145, $C$2:$C$620, C145, $D$2:$D$620, D145, $E$2:$E$620, E145) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -8233,7 +8233,7 @@
         <v>646</v>
       </c>
       <c r="N146" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B146, $C$2:$C$620, C146, $D$2:$D$620, D146, $E$2:$E$620, E146) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
       <c r="O146" s="35" t="s">
@@ -8282,7 +8282,7 @@
         <v>650</v>
       </c>
       <c r="N147" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B147, $C$2:$C$620, C147, $D$2:$D$620, D147, $E$2:$E$620, E147) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -8328,7 +8328,7 @@
         <v>400</v>
       </c>
       <c r="N148" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B148, $C$2:$C$620, C148, $D$2:$D$620, D148, $E$2:$E$620, E148) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -8362,7 +8362,7 @@
       </c>
       <c r="J149" s="32"/>
       <c r="N149" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B149, $C$2:$C$620, C149, $D$2:$D$620, D149, $E$2:$E$620, E149) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
       <c r="O149" s="22"/>
@@ -8405,11 +8405,11 @@
         <v>16500</v>
       </c>
       <c r="M150" s="17">
-        <f>ABS((D150*E150)-L150)</f>
+        <f t="shared" ref="M150:M158" si="8">ABS((D150*E150)-L150)</f>
         <v>1400</v>
       </c>
       <c r="N150" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B150, $C$2:$C$620, C150, $D$2:$D$620, D150, $E$2:$E$620, E150) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
       <c r="O150" s="35" t="s">
@@ -8454,11 +8454,11 @@
         <v>39300</v>
       </c>
       <c r="M151" s="17">
-        <f>ABS((D151*E151)-L151)</f>
+        <f t="shared" si="8"/>
         <v>18350</v>
       </c>
       <c r="N151" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B151, $C$2:$C$620, C151, $D$2:$D$620, D151, $E$2:$E$620, E151) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -8500,11 +8500,11 @@
         <v>18800</v>
       </c>
       <c r="M152" s="17">
-        <f>ABS((D152*E152)-L152)</f>
+        <f t="shared" si="8"/>
         <v>500</v>
       </c>
       <c r="N152" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B152, $C$2:$C$620, C152, $D$2:$D$620, D152, $E$2:$E$620, E152) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
       <c r="O152" s="36" t="s">
@@ -8549,11 +8549,11 @@
         <v>7578</v>
       </c>
       <c r="M153" s="25">
-        <f>ABS((D153*E153)-L153)</f>
+        <f t="shared" si="8"/>
         <v>294</v>
       </c>
       <c r="N153" s="26" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B153, $C$2:$C$620, C153, $D$2:$D$620, D153, $E$2:$E$620, E153) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Duplicate</v>
       </c>
     </row>
@@ -8595,11 +8595,11 @@
         <v>7578</v>
       </c>
       <c r="M154" s="25">
-        <f>ABS((D154*E154)-L154)</f>
+        <f t="shared" si="8"/>
         <v>294</v>
       </c>
       <c r="N154" s="27" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B154, $C$2:$C$620, C154, $D$2:$D$620, D154, $E$2:$E$620, E154) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Duplicate</v>
       </c>
     </row>
@@ -8641,11 +8641,11 @@
         <v>4968</v>
       </c>
       <c r="M155" s="25">
-        <f>ABS((D155*E155)-L155)</f>
+        <f t="shared" si="8"/>
         <v>280</v>
       </c>
       <c r="N155" s="27" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B155, $C$2:$C$620, C155, $D$2:$D$620, D155, $E$2:$E$620, E155) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
       <c r="O155" s="27"/>
@@ -8689,11 +8689,11 @@
         <v>8820</v>
       </c>
       <c r="M156" s="25">
-        <f>ABS((D156*E156)-L156)</f>
+        <f t="shared" si="8"/>
         <v>650</v>
       </c>
       <c r="N156" s="27" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B156, $C$2:$C$620, C156, $D$2:$D$620, D156, $E$2:$E$620, E156) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
       <c r="O156" s="27"/>
@@ -8737,11 +8737,11 @@
         <v>36946</v>
       </c>
       <c r="M157" s="25">
-        <f>ABS((D157*E157)-L157)</f>
+        <f t="shared" si="8"/>
         <v>934</v>
       </c>
       <c r="N157" s="27" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B157, $C$2:$C$620, C157, $D$2:$D$620, D157, $E$2:$E$620, E157) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
       <c r="O157" s="27"/>
@@ -8785,11 +8785,11 @@
         <v>11360</v>
       </c>
       <c r="M158" s="17">
-        <f>ABS((D158*E158)-L158)</f>
+        <f t="shared" si="8"/>
         <v>300</v>
       </c>
       <c r="N158" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B158, $C$2:$C$620, C158, $D$2:$D$620, D158, $E$2:$E$620, E158) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -8825,7 +8825,7 @@
         <v>117</v>
       </c>
       <c r="N159" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B159, $C$2:$C$620, C159, $D$2:$D$620, D159, $E$2:$E$620, E159) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
       <c r="O159" s="35" t="s">
@@ -8874,7 +8874,7 @@
         <v>300</v>
       </c>
       <c r="N160" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B160, $C$2:$C$620, C160, $D$2:$D$620, D160, $E$2:$E$620, E160) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -8920,7 +8920,7 @@
         <v>650</v>
       </c>
       <c r="N161" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B161, $C$2:$C$620, C161, $D$2:$D$620, D161, $E$2:$E$620, E161) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -8954,7 +8954,7 @@
       </c>
       <c r="J162" s="32"/>
       <c r="N162" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B162, $C$2:$C$620, C162, $D$2:$D$620, D162, $E$2:$E$620, E162) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
       <c r="O162" s="35" t="s">
@@ -9004,7 +9004,7 @@
         <v>654.5</v>
       </c>
       <c r="N163" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B163, $C$2:$C$620, C163, $D$2:$D$620, D163, $E$2:$E$620, E163) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
       <c r="O163" s="35" t="s">
@@ -9043,7 +9043,7 @@
         <v>117</v>
       </c>
       <c r="N164" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B164, $C$2:$C$620, C164, $D$2:$D$620, D164, $E$2:$E$620, E164) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -9089,7 +9089,7 @@
         <v>300</v>
       </c>
       <c r="N165" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B165, $C$2:$C$620, C165, $D$2:$D$620, D165, $E$2:$E$620, E165) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -9135,7 +9135,7 @@
         <v>11409.000000000004</v>
       </c>
       <c r="N166" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B166, $C$2:$C$620, C166, $D$2:$D$620, D166, $E$2:$E$620, E166) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
       <c r="P166"/>
@@ -9182,7 +9182,7 @@
         <v>34175</v>
       </c>
       <c r="N167" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B167, $C$2:$C$620, C167, $D$2:$D$620, D167, $E$2:$E$620, E167) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -9218,7 +9218,7 @@
         <v>117</v>
       </c>
       <c r="N168" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B168, $C$2:$C$620, C168, $D$2:$D$620, D168, $E$2:$E$620, E168) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -9264,7 +9264,7 @@
         <v>800</v>
       </c>
       <c r="N169" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B169, $C$2:$C$620, C169, $D$2:$D$620, D169, $E$2:$E$620, E169) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -9310,7 +9310,7 @@
         <v>265</v>
       </c>
       <c r="N170" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B170, $C$2:$C$620, C170, $D$2:$D$620, D170, $E$2:$E$620, E170) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -9356,7 +9356,7 @@
         <v>300</v>
       </c>
       <c r="N171" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B171, $C$2:$C$620, C171, $D$2:$D$620, D171, $E$2:$E$620, E171) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -9392,7 +9392,7 @@
         <v>116</v>
       </c>
       <c r="N172" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B172, $C$2:$C$620, C172, $D$2:$D$620, D172, $E$2:$E$620, E172) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -9438,7 +9438,7 @@
         <v>270</v>
       </c>
       <c r="N173" s="27" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B173, $C$2:$C$620, C173, $D$2:$D$620, D173, $E$2:$E$620, E173) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
       <c r="O173" s="36" t="s">
@@ -9487,7 +9487,7 @@
         <v>188.60000000000014</v>
       </c>
       <c r="N174" s="27" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B174, $C$2:$C$620, C174, $D$2:$D$620, D174, $E$2:$E$620, E174) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
       <c r="O174" s="36" t="s">
@@ -9536,7 +9536,7 @@
         <v>1000</v>
       </c>
       <c r="N175" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B175, $C$2:$C$620, C175, $D$2:$D$620, D175, $E$2:$E$620, E175) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
       <c r="P175" s="27"/>
@@ -9573,7 +9573,7 @@
         <v>54</v>
       </c>
       <c r="N176" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B176, $C$2:$C$620, C176, $D$2:$D$620, D176, $E$2:$E$620, E176) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -9619,7 +9619,7 @@
         <v>650</v>
       </c>
       <c r="N177" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B177, $C$2:$C$620, C177, $D$2:$D$620, D177, $E$2:$E$620, E177) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
       <c r="O177" s="27"/>
@@ -9666,7 +9666,7 @@
         <v>1450</v>
       </c>
       <c r="N178" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B178, $C$2:$C$620, C178, $D$2:$D$620, D178, $E$2:$E$620, E178) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -9712,7 +9712,7 @@
         <v>260</v>
       </c>
       <c r="N179" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B179, $C$2:$C$620, C179, $D$2:$D$620, D179, $E$2:$E$620, E179) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -9748,7 +9748,7 @@
         <v>116</v>
       </c>
       <c r="N180" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B180, $C$2:$C$620, C180, $D$2:$D$620, D180, $E$2:$E$620, E180) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -9787,7 +9787,7 @@
       <c r="L181" s="16"/>
       <c r="M181" s="16"/>
       <c r="N181" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B181, $C$2:$C$620, C181, $D$2:$D$620, D181, $E$2:$E$620, E181) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
       <c r="O181" s="36" t="s">
@@ -9837,7 +9837,7 @@
         <v>656.5</v>
       </c>
       <c r="N182" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B182, $C$2:$C$620, C182, $D$2:$D$620, D182, $E$2:$E$620, E182) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -9883,7 +9883,7 @@
         <v>268</v>
       </c>
       <c r="N183" s="52" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B183, $C$2:$C$620, C183, $D$2:$D$620, D183, $E$2:$E$620, E183) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
       <c r="O183" s="22"/>
@@ -9926,7 +9926,7 @@
       <c r="L184" s="17"/>
       <c r="M184" s="17"/>
       <c r="N184" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B184, $C$2:$C$620, C184, $D$2:$D$620, D184, $E$2:$E$620, E184) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
       <c r="O184" s="10"/>
@@ -9974,7 +9974,7 @@
         <v>14149.000000000004</v>
       </c>
       <c r="N185" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B185, $C$2:$C$620, C185, $D$2:$D$620, D185, $E$2:$E$620, E185) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
       <c r="P185"/>
@@ -10021,7 +10021,7 @@
         <v>300</v>
       </c>
       <c r="N186" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B186, $C$2:$C$620, C186, $D$2:$D$620, D186, $E$2:$E$620, E186) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
       <c r="O186" s="35" t="s">
@@ -10070,7 +10070,7 @@
         <v>940</v>
       </c>
       <c r="N187" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B187, $C$2:$C$620, C187, $D$2:$D$620, D187, $E$2:$E$620, E187) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -10107,7 +10107,7 @@
       <c r="L188" s="17"/>
       <c r="M188" s="17"/>
       <c r="N188" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B188, $C$2:$C$620, C188, $D$2:$D$620, D188, $E$2:$E$620, E188) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
       <c r="O188" s="10"/>
@@ -10155,7 +10155,7 @@
         <v>300</v>
       </c>
       <c r="N189" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B189, $C$2:$C$620, C189, $D$2:$D$620, D189, $E$2:$E$620, E189) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -10191,7 +10191,7 @@
         <v>117</v>
       </c>
       <c r="N190" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B190, $C$2:$C$620, C190, $D$2:$D$620, D190, $E$2:$E$620, E190) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -10225,7 +10225,7 @@
       </c>
       <c r="J191" s="32"/>
       <c r="N191" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B191, $C$2:$C$620, C191, $D$2:$D$620, D191, $E$2:$E$620, E191) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
     </row>
@@ -10261,7 +10261,7 @@
         <v>117</v>
       </c>
       <c r="N192" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B192, $C$2:$C$620, C192, $D$2:$D$620, D192, $E$2:$E$620, E192) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
       <c r="O192" s="27"/>
@@ -10308,7 +10308,7 @@
         <v>902.5</v>
       </c>
       <c r="N193" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B193, $C$2:$C$620, C193, $D$2:$D$620, D193, $E$2:$E$620, E193) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="7"/>
         <v>Unique</v>
       </c>
       <c r="O193" s="10"/>
@@ -10356,7 +10356,7 @@
         <v>350</v>
       </c>
       <c r="N194" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B194, $C$2:$C$620, C194, $D$2:$D$620, D194, $E$2:$E$620, E194) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" ref="N194:N257" si="9">IF(COUNTIFS( $B$2:$B$620, B194, $C$2:$C$620, C194, $D$2:$D$620, D194, $E$2:$E$620, E194) &gt; 1, "Duplicate", "Unique")</f>
         <v>Unique</v>
       </c>
       <c r="O194" s="10"/>
@@ -10394,7 +10394,7 @@
         <v>116</v>
       </c>
       <c r="N195" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B195, $C$2:$C$620, C195, $D$2:$D$620, D195, $E$2:$E$620, E195) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -10431,7 +10431,7 @@
       <c r="L196" s="17"/>
       <c r="M196" s="17"/>
       <c r="N196" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B196, $C$2:$C$620, C196, $D$2:$D$620, D196, $E$2:$E$620, E196) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="O196" s="10"/>
@@ -10478,7 +10478,7 @@
         <v>250</v>
       </c>
       <c r="N197" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B197, $C$2:$C$620, C197, $D$2:$D$620, D197, $E$2:$E$620, E197) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -10515,7 +10515,7 @@
       <c r="L198" s="17"/>
       <c r="M198" s="17"/>
       <c r="N198" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B198, $C$2:$C$620, C198, $D$2:$D$620, D198, $E$2:$E$620, E198) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="O198" s="10"/>
@@ -10563,7 +10563,7 @@
         <v>501</v>
       </c>
       <c r="N199" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B199, $C$2:$C$620, C199, $D$2:$D$620, D199, $E$2:$E$620, E199) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="O199" s="35" t="s">
@@ -10613,7 +10613,7 @@
         <v>376</v>
       </c>
       <c r="N200" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B200, $C$2:$C$620, C200, $D$2:$D$620, D200, $E$2:$E$620, E200) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -10649,7 +10649,7 @@
         <v>117</v>
       </c>
       <c r="N201" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B201, $C$2:$C$620, C201, $D$2:$D$620, D201, $E$2:$E$620, E201) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -10695,7 +10695,7 @@
         <v>650</v>
       </c>
       <c r="N202" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B202, $C$2:$C$620, C202, $D$2:$D$620, D202, $E$2:$E$620, E202) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="P202" s="27"/>
@@ -10735,7 +10735,7 @@
       <c r="L203" s="17"/>
       <c r="M203" s="17"/>
       <c r="N203" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B203, $C$2:$C$620, C203, $D$2:$D$620, D203, $E$2:$E$620, E203) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="O203" s="10"/>
@@ -10783,7 +10783,7 @@
         <v>290</v>
       </c>
       <c r="N204" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B204, $C$2:$C$620, C204, $D$2:$D$620, D204, $E$2:$E$620, E204) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="O204" s="10"/>
@@ -10831,7 +10831,7 @@
         <v>250</v>
       </c>
       <c r="N205" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B205, $C$2:$C$620, C205, $D$2:$D$620, D205, $E$2:$E$620, E205) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -10877,7 +10877,7 @@
         <v>300</v>
       </c>
       <c r="N206" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B206, $C$2:$C$620, C206, $D$2:$D$620, D206, $E$2:$E$620, E206) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -10923,7 +10923,7 @@
         <v>320</v>
       </c>
       <c r="N207" s="27" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B207, $C$2:$C$620, C207, $D$2:$D$620, D207, $E$2:$E$620, E207) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="O207" s="27"/>
@@ -10971,7 +10971,7 @@
         <v>448</v>
       </c>
       <c r="N208" s="26" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B208, $C$2:$C$620, C208, $D$2:$D$620, D208, $E$2:$E$620, E208) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="O208" s="27"/>
@@ -11009,7 +11009,7 @@
         <v>116</v>
       </c>
       <c r="N209" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B209, $C$2:$C$620, C209, $D$2:$D$620, D209, $E$2:$E$620, E209) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="P209" s="27"/>
@@ -11052,11 +11052,11 @@
         <v>9320</v>
       </c>
       <c r="M210" s="17">
-        <f>ABS((D210*E210)-L210)</f>
+        <f t="shared" ref="M210:M218" si="10">ABS((D210*E210)-L210)</f>
         <v>650</v>
       </c>
       <c r="N210" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B210, $C$2:$C$620, C210, $D$2:$D$620, D210, $E$2:$E$620, E210) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="P210" s="27"/>
@@ -11099,11 +11099,11 @@
         <v>2896</v>
       </c>
       <c r="M211" s="17">
-        <f>ABS((D211*E211)-L211)</f>
+        <f t="shared" si="10"/>
         <v>276</v>
       </c>
       <c r="N211" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B211, $C$2:$C$620, C211, $D$2:$D$620, D211, $E$2:$E$620, E211) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -11145,11 +11145,11 @@
         <v>5520</v>
       </c>
       <c r="M212" s="25">
-        <f>ABS((D212*E212)-L212)</f>
+        <f t="shared" si="10"/>
         <v>300</v>
       </c>
       <c r="N212" s="26" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B212, $C$2:$C$620, C212, $D$2:$D$620, D212, $E$2:$E$620, E212) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="O212" s="35" t="s">
@@ -11194,11 +11194,11 @@
         <v>2657</v>
       </c>
       <c r="M213" s="25">
-        <f>ABS((D213*E213)-L213)</f>
+        <f t="shared" si="10"/>
         <v>253</v>
       </c>
       <c r="N213" s="27" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B213, $C$2:$C$620, C213, $D$2:$D$620, D213, $E$2:$E$620, E213) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Duplicate</v>
       </c>
       <c r="O213" s="35" t="s">
@@ -11243,11 +11243,11 @@
         <v>2554.5</v>
       </c>
       <c r="M214" s="25">
-        <f>ABS((D214*E214)-L214)</f>
+        <f t="shared" si="10"/>
         <v>355.5</v>
       </c>
       <c r="N214" s="27" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B214, $C$2:$C$620, C214, $D$2:$D$620, D214, $E$2:$E$620, E214) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Duplicate</v>
       </c>
       <c r="O214" s="35" t="s">
@@ -11292,11 +11292,11 @@
         <v>5585</v>
       </c>
       <c r="M215" s="25">
-        <f>ABS((D215*E215)-L215)</f>
+        <f t="shared" si="10"/>
         <v>395</v>
       </c>
       <c r="N215" s="27" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B215, $C$2:$C$620, C215, $D$2:$D$620, D215, $E$2:$E$620, E215) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Duplicate</v>
       </c>
       <c r="O215" s="35" t="s">
@@ -11341,11 +11341,11 @@
         <v>5730</v>
       </c>
       <c r="M216" s="25">
-        <f>ABS((D216*E216)-L216)</f>
+        <f t="shared" si="10"/>
         <v>250</v>
       </c>
       <c r="N216" s="27" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B216, $C$2:$C$620, C216, $D$2:$D$620, D216, $E$2:$E$620, E216) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Duplicate</v>
       </c>
       <c r="O216" s="35" t="s">
@@ -11391,11 +11391,11 @@
         <v>11175</v>
       </c>
       <c r="M217" s="25">
-        <f>ABS((D217*E217)-L217)</f>
+        <f t="shared" si="10"/>
         <v>300</v>
       </c>
       <c r="N217" s="27" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B217, $C$2:$C$620, C217, $D$2:$D$620, D217, $E$2:$E$620, E217) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="O217" s="27"/>
@@ -11439,11 +11439,11 @@
         <v>4402</v>
       </c>
       <c r="M218" s="25">
-        <f>ABS((D218*E218)-L218)</f>
+        <f t="shared" si="10"/>
         <v>188</v>
       </c>
       <c r="N218" s="27" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B218, $C$2:$C$620, C218, $D$2:$D$620, D218, $E$2:$E$620, E218) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="O218" s="27"/>
@@ -11484,7 +11484,7 @@
       <c r="L219" s="16"/>
       <c r="M219" s="16"/>
       <c r="N219" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B219, $C$2:$C$620, C219, $D$2:$D$620, D219, $E$2:$E$620, E219) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="O219"/>
@@ -11521,7 +11521,7 @@
         <v>117</v>
       </c>
       <c r="N220" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B220, $C$2:$C$620, C220, $D$2:$D$620, D220, $E$2:$E$620, E220) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="O220" s="27"/>
@@ -11568,7 +11568,7 @@
         <v>360</v>
       </c>
       <c r="N221" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B221, $C$2:$C$620, C221, $D$2:$D$620, D221, $E$2:$E$620, E221) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -11602,7 +11602,7 @@
       </c>
       <c r="J222" s="32"/>
       <c r="N222" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B222, $C$2:$C$620, C222, $D$2:$D$620, D222, $E$2:$E$620, E222) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -11648,7 +11648,7 @@
         <v>275</v>
       </c>
       <c r="N223" s="27" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B223, $C$2:$C$620, C223, $D$2:$D$620, D223, $E$2:$E$620, E223) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Duplicate</v>
       </c>
     </row>
@@ -11694,7 +11694,7 @@
         <v>225</v>
       </c>
       <c r="N224" s="27" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B224, $C$2:$C$620, C224, $D$2:$D$620, D224, $E$2:$E$620, E224) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Duplicate</v>
       </c>
     </row>
@@ -11740,7 +11740,7 @@
         <v>500</v>
       </c>
       <c r="N225" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B225, $C$2:$C$620, C225, $D$2:$D$620, D225, $E$2:$E$620, E225) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -11786,7 +11786,7 @@
         <v>527.5</v>
       </c>
       <c r="N226" s="27" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B226, $C$2:$C$620, C226, $D$2:$D$620, D226, $E$2:$E$620, E226) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="O226" s="27"/>
@@ -11829,7 +11829,7 @@
       <c r="L227" s="25"/>
       <c r="M227" s="25"/>
       <c r="N227" s="27" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B227, $C$2:$C$620, C227, $D$2:$D$620, D227, $E$2:$E$620, E227) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="O227" s="27"/>
@@ -11877,7 +11877,7 @@
         <v>1000</v>
       </c>
       <c r="N228" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B228, $C$2:$C$620, C228, $D$2:$D$620, D228, $E$2:$E$620, E228) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -11913,7 +11913,7 @@
         <v>116</v>
       </c>
       <c r="N229" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B229, $C$2:$C$620, C229, $D$2:$D$620, D229, $E$2:$E$620, E229) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -11959,7 +11959,7 @@
         <v>300</v>
       </c>
       <c r="N230" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B230, $C$2:$C$620, C230, $D$2:$D$620, D230, $E$2:$E$620, E230) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12005,7 +12005,7 @@
         <v>300</v>
       </c>
       <c r="N231" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B231, $C$2:$C$620, C231, $D$2:$D$620, D231, $E$2:$E$620, E231) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12044,7 +12044,7 @@
       <c r="L232" s="16"/>
       <c r="M232" s="16"/>
       <c r="N232" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B232, $C$2:$C$620, C232, $D$2:$D$620, D232, $E$2:$E$620, E232) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12080,7 +12080,7 @@
         <v>116</v>
       </c>
       <c r="N233" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B233, $C$2:$C$620, C233, $D$2:$D$620, D233, $E$2:$E$620, E233) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12126,7 +12126,7 @@
         <v>300</v>
       </c>
       <c r="N234" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B234, $C$2:$C$620, C234, $D$2:$D$620, D234, $E$2:$E$620, E234) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12172,7 +12172,7 @@
         <v>400</v>
       </c>
       <c r="N235" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B235, $C$2:$C$620, C235, $D$2:$D$620, D235, $E$2:$E$620, E235) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12218,7 +12218,7 @@
         <v>500</v>
       </c>
       <c r="N236" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B236, $C$2:$C$620, C236, $D$2:$D$620, D236, $E$2:$E$620, E236) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12257,7 +12257,7 @@
       <c r="L237" s="17"/>
       <c r="M237" s="17"/>
       <c r="N237" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B237, $C$2:$C$620, C237, $D$2:$D$620, D237, $E$2:$E$620, E237) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="O237" s="10"/>
@@ -12293,7 +12293,7 @@
       </c>
       <c r="J238" s="32"/>
       <c r="N238" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B238, $C$2:$C$620, C238, $D$2:$D$620, D238, $E$2:$E$620, E238) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12339,7 +12339,7 @@
         <v>480</v>
       </c>
       <c r="N239" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B239, $C$2:$C$620, C239, $D$2:$D$620, D239, $E$2:$E$620, E239) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="O239" s="10"/>
@@ -12387,7 +12387,7 @@
         <v>800</v>
       </c>
       <c r="N240" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B240, $C$2:$C$620, C240, $D$2:$D$620, D240, $E$2:$E$620, E240) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="O240" s="35" t="s">
@@ -12436,7 +12436,7 @@
         <v>300</v>
       </c>
       <c r="N241" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B241, $C$2:$C$620, C241, $D$2:$D$620, D241, $E$2:$E$620, E241) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12482,7 +12482,7 @@
         <v>500</v>
       </c>
       <c r="N242" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B242, $C$2:$C$620, C242, $D$2:$D$620, D242, $E$2:$E$620, E242) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12528,7 +12528,7 @@
         <v>260</v>
       </c>
       <c r="N243" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B243, $C$2:$C$620, C243, $D$2:$D$620, D243, $E$2:$E$620, E243) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12567,7 +12567,7 @@
       <c r="L244" s="16"/>
       <c r="M244" s="16"/>
       <c r="N244" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B244, $C$2:$C$620, C244, $D$2:$D$620, D244, $E$2:$E$620, E244) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="P244" s="22"/>
@@ -12604,7 +12604,7 @@
         <v>117</v>
       </c>
       <c r="N245" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B245, $C$2:$C$620, C245, $D$2:$D$620, D245, $E$2:$E$620, E245) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12638,7 +12638,7 @@
       </c>
       <c r="J246" s="32"/>
       <c r="N246" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B246, $C$2:$C$620, C246, $D$2:$D$620, D246, $E$2:$E$620, E246) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12684,7 +12684,7 @@
         <v>275</v>
       </c>
       <c r="N247" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B247, $C$2:$C$620, C247, $D$2:$D$620, D247, $E$2:$E$620, E247) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12730,7 +12730,7 @@
         <v>140</v>
       </c>
       <c r="N248" s="27" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B248, $C$2:$C$620, C248, $D$2:$D$620, D248, $E$2:$E$620, E248) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Duplicate</v>
       </c>
       <c r="P248" s="27"/>
@@ -12777,7 +12777,7 @@
         <v>300</v>
       </c>
       <c r="N249" s="27" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B249, $C$2:$C$620, C249, $D$2:$D$620, D249, $E$2:$E$620, E249) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Duplicate</v>
       </c>
     </row>
@@ -12823,7 +12823,7 @@
         <v>271.80000000000018</v>
       </c>
       <c r="N250" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B250, $C$2:$C$620, C250, $D$2:$D$620, D250, $E$2:$E$620, E250) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12862,7 +12862,7 @@
         <v>143</v>
       </c>
       <c r="N251" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B251, $C$2:$C$620, C251, $D$2:$D$620, D251, $E$2:$E$620, E251) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12896,7 +12896,7 @@
       </c>
       <c r="J252" s="32"/>
       <c r="N252" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B252, $C$2:$C$620, C252, $D$2:$D$620, D252, $E$2:$E$620, E252) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -12942,7 +12942,7 @@
         <v>370</v>
       </c>
       <c r="N253" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B253, $C$2:$C$620, C253, $D$2:$D$620, D253, $E$2:$E$620, E253) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="P253" s="27"/>
@@ -12979,7 +12979,7 @@
         <v>116</v>
       </c>
       <c r="N254" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B254, $C$2:$C$620, C254, $D$2:$D$620, D254, $E$2:$E$620, E254) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13015,7 +13015,7 @@
         <v>117</v>
       </c>
       <c r="N255" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B255, $C$2:$C$620, C255, $D$2:$D$620, D255, $E$2:$E$620, E255) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13057,11 +13057,11 @@
         <v>14400</v>
       </c>
       <c r="M256" s="17">
-        <f>ABS((D256*E256)-L256)</f>
+        <f t="shared" ref="M256:M261" si="11">ABS((D256*E256)-L256)</f>
         <v>500</v>
       </c>
       <c r="N256" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B256, $C$2:$C$620, C256, $D$2:$D$620, D256, $E$2:$E$620, E256) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13103,11 +13103,11 @@
         <v>14552</v>
       </c>
       <c r="M257" s="17">
-        <f>ABS((D257*E257)-L257)</f>
+        <f t="shared" si="11"/>
         <v>300</v>
       </c>
       <c r="N257" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B257, $C$2:$C$620, C257, $D$2:$D$620, D257, $E$2:$E$620, E257) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="9"/>
         <v>Unique</v>
       </c>
       <c r="O257" s="35" t="s">
@@ -13153,11 +13153,11 @@
         <v>6105</v>
       </c>
       <c r="M258" s="25">
-        <f>ABS((D258*E258)-L258)</f>
+        <f t="shared" si="11"/>
         <v>150</v>
       </c>
       <c r="N258" s="26" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B258, $C$2:$C$620, C258, $D$2:$D$620, D258, $E$2:$E$620, E258) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" ref="N258:N325" si="12">IF(COUNTIFS( $B$2:$B$620, B258, $C$2:$C$620, C258, $D$2:$D$620, D258, $E$2:$E$620, E258) &gt; 1, "Duplicate", "Unique")</f>
         <v>Duplicate</v>
       </c>
     </row>
@@ -13199,11 +13199,11 @@
         <v>6005</v>
       </c>
       <c r="M259" s="25">
-        <f>ABS((D259*E259)-L259)</f>
+        <f t="shared" si="11"/>
         <v>250</v>
       </c>
       <c r="N259" s="27" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B259, $C$2:$C$620, C259, $D$2:$D$620, D259, $E$2:$E$620, E259) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Duplicate</v>
       </c>
     </row>
@@ -13245,11 +13245,11 @@
         <v>15300</v>
       </c>
       <c r="M260" s="17">
-        <f>ABS((D260*E260)-L260)</f>
+        <f t="shared" si="11"/>
         <v>420</v>
       </c>
       <c r="N260" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B260, $C$2:$C$620, C260, $D$2:$D$620, D260, $E$2:$E$620, E260) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13291,11 +13291,11 @@
         <v>4260</v>
       </c>
       <c r="M261" s="17">
-        <f>ABS((D261*E261)-L261)</f>
+        <f t="shared" si="11"/>
         <v>250</v>
       </c>
       <c r="N261" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B261, $C$2:$C$620, C261, $D$2:$D$620, D261, $E$2:$E$620, E261) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
       <c r="P261" s="27"/>
@@ -13330,7 +13330,7 @@
       </c>
       <c r="J262" s="32"/>
       <c r="N262" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B262, $C$2:$C$620, C262, $D$2:$D$620, D262, $E$2:$E$620, E262) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13376,7 +13376,7 @@
         <v>816</v>
       </c>
       <c r="N263" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B263, $C$2:$C$620, C263, $D$2:$D$620, D263, $E$2:$E$620, E263) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13422,7 +13422,7 @@
         <v>280</v>
       </c>
       <c r="N264" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B264, $C$2:$C$620, C264, $D$2:$D$620, D264, $E$2:$E$620, E264) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13456,7 +13456,7 @@
       </c>
       <c r="J265" s="32"/>
       <c r="N265" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B265, $C$2:$C$620, C265, $D$2:$D$620, D265, $E$2:$E$620, E265) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
       <c r="P265" s="27"/>
@@ -13491,7 +13491,7 @@
       </c>
       <c r="J266" s="32"/>
       <c r="N266" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B266, $C$2:$C$620, C266, $D$2:$D$620, D266, $E$2:$E$620, E266) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
       <c r="O266" s="27"/>
@@ -13538,7 +13538,7 @@
         <v>300</v>
       </c>
       <c r="N267" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B267, $C$2:$C$620, C267, $D$2:$D$620, D267, $E$2:$E$620, E267) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13572,7 +13572,7 @@
       </c>
       <c r="J268" s="32"/>
       <c r="N268" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B268, $C$2:$C$620, C268, $D$2:$D$620, D268, $E$2:$E$620, E268) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
       <c r="P268" s="27"/>
@@ -13619,7 +13619,7 @@
         <v>450</v>
       </c>
       <c r="N269" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B269, $C$2:$C$620, C269, $D$2:$D$620, D269, $E$2:$E$620, E269) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13655,7 +13655,7 @@
         <v>116</v>
       </c>
       <c r="N270" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B270, $C$2:$C$620, C270, $D$2:$D$620, D270, $E$2:$E$620, E270) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13701,7 +13701,7 @@
         <v>48320</v>
       </c>
       <c r="N271" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B271, $C$2:$C$620, C271, $D$2:$D$620, D271, $E$2:$E$620, E271) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
       <c r="O271" s="35" t="s">
@@ -13740,7 +13740,7 @@
         <v>117</v>
       </c>
       <c r="N272" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B272, $C$2:$C$620, C272, $D$2:$D$620, D272, $E$2:$E$620, E272) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13786,7 +13786,7 @@
         <v>290</v>
       </c>
       <c r="N273" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B273, $C$2:$C$620, C273, $D$2:$D$620, D273, $E$2:$E$620, E273) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13820,7 +13820,7 @@
       </c>
       <c r="J274" s="32"/>
       <c r="N274" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B274, $C$2:$C$620, C274, $D$2:$D$620, D274, $E$2:$E$620, E274) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13866,7 +13866,7 @@
         <v>1800</v>
       </c>
       <c r="N275" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B275, $C$2:$C$620, C275, $D$2:$D$620, D275, $E$2:$E$620, E275) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13902,7 +13902,7 @@
         <v>116</v>
       </c>
       <c r="N276" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B276, $C$2:$C$620, C276, $D$2:$D$620, D276, $E$2:$E$620, E276) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13948,7 +13948,7 @@
         <v>300</v>
       </c>
       <c r="N277" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B277, $C$2:$C$620, C277, $D$2:$D$620, D277, $E$2:$E$620, E277) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -13984,7 +13984,7 @@
         <v>116</v>
       </c>
       <c r="N278" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B278, $C$2:$C$620, C278, $D$2:$D$620, D278, $E$2:$E$620, E278) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -14030,7 +14030,7 @@
         <v>47900</v>
       </c>
       <c r="N279" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B279, $C$2:$C$620, C279, $D$2:$D$620, D279, $E$2:$E$620, E279) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
       <c r="O279" s="35" t="s">
@@ -14079,7 +14079,7 @@
         <v>650</v>
       </c>
       <c r="N280" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B280, $C$2:$C$620, C280, $D$2:$D$620, D280, $E$2:$E$620, E280) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
       <c r="O280" s="35" t="s">
@@ -14128,7 +14128,7 @@
         <v>495</v>
       </c>
       <c r="N281" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B281, $C$2:$C$620, C281, $D$2:$D$620, D281, $E$2:$E$620, E281) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
       <c r="O281" s="35" t="s">
@@ -14177,7 +14177,7 @@
         <v>450</v>
       </c>
       <c r="N282" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B282, $C$2:$C$620, C282, $D$2:$D$620, D282, $E$2:$E$620, E282) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -14213,7 +14213,7 @@
         <v>116</v>
       </c>
       <c r="N283" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B283, $C$2:$C$620, C283, $D$2:$D$620, D283, $E$2:$E$620, E283) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -14247,7 +14247,7 @@
       </c>
       <c r="J284" s="32"/>
       <c r="N284" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B284, $C$2:$C$620, C284, $D$2:$D$620, D284, $E$2:$E$620, E284) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -14293,7 +14293,7 @@
         <v>300</v>
       </c>
       <c r="N285" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B285, $C$2:$C$620, C285, $D$2:$D$620, D285, $E$2:$E$620, E285) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
       <c r="O285" s="35" t="s">
@@ -14331,7 +14331,7 @@
       </c>
       <c r="J286" s="32"/>
       <c r="N286" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B286, $C$2:$C$620, C286, $D$2:$D$620, D286, $E$2:$E$620, E286) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -14370,7 +14370,7 @@
       <c r="L287" s="16"/>
       <c r="M287" s="16"/>
       <c r="N287" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B287, $C$2:$C$620, C287, $D$2:$D$620, D287, $E$2:$E$620, E287) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
       <c r="O287"/>
@@ -14407,7 +14407,7 @@
         <v>116</v>
       </c>
       <c r="N288" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B288, $C$2:$C$620, C288, $D$2:$D$620, D288, $E$2:$E$620, E288) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -14453,7 +14453,7 @@
         <v>650</v>
       </c>
       <c r="N289" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B289, $C$2:$C$620, C289, $D$2:$D$620, D289, $E$2:$E$620, E289) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
       <c r="O289"/>
@@ -14501,7 +14501,7 @@
         <v>300</v>
       </c>
       <c r="N290" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B290, $C$2:$C$620, C290, $D$2:$D$620, D290, $E$2:$E$620, E290) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -14537,7 +14537,7 @@
         <v>116</v>
       </c>
       <c r="N291" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B291, $C$2:$C$620, C291, $D$2:$D$620, D291, $E$2:$E$620, E291) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -14583,7 +14583,7 @@
         <v>47480</v>
       </c>
       <c r="N292" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B292, $C$2:$C$620, C292, $D$2:$D$620, D292, $E$2:$E$620, E292) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -14629,7 +14629,7 @@
         <v>340</v>
       </c>
       <c r="N293" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B293, $C$2:$C$620, C293, $D$2:$D$620, D293, $E$2:$E$620, E293) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -14665,7 +14665,7 @@
         <v>116</v>
       </c>
       <c r="N294" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B294, $C$2:$C$620, C294, $D$2:$D$620, D294, $E$2:$E$620, E294) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -14711,7 +14711,7 @@
         <v>285</v>
       </c>
       <c r="N295" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B295, $C$2:$C$620, C295, $D$2:$D$620, D295, $E$2:$E$620, E295) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -14757,7 +14757,7 @@
         <v>726</v>
       </c>
       <c r="N296" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B296, $C$2:$C$620, C296, $D$2:$D$620, D296, $E$2:$E$620, E296) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -14791,7 +14791,7 @@
       </c>
       <c r="J297" s="32"/>
       <c r="N297" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B297, $C$2:$C$620, C297, $D$2:$D$620, D297, $E$2:$E$620, E297) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -14837,7 +14837,7 @@
         <v>300</v>
       </c>
       <c r="N298" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B298, $C$2:$C$620, C298, $D$2:$D$620, D298, $E$2:$E$620, E298) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -14871,7 +14871,7 @@
       </c>
       <c r="J299" s="32"/>
       <c r="N299" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B299, $C$2:$C$620, C299, $D$2:$D$620, D299, $E$2:$E$620, E299) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -14907,7 +14907,7 @@
         <v>117</v>
       </c>
       <c r="N300" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B300, $C$2:$C$620, C300, $D$2:$D$620, D300, $E$2:$E$620, E300) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -14953,7 +14953,7 @@
         <v>300</v>
       </c>
       <c r="N301" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B301, $C$2:$C$620, C301, $D$2:$D$620, D301, $E$2:$E$620, E301) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -14994,7 +14994,7 @@
       <c r="L302" s="16"/>
       <c r="M302" s="16"/>
       <c r="N302" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B302, $C$2:$C$620, C302, $D$2:$D$620, D302, $E$2:$E$620, E302) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -15040,7 +15040,7 @@
         <v>275</v>
       </c>
       <c r="N303" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B303, $C$2:$C$620, C303, $D$2:$D$620, D303, $E$2:$E$620, E303) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -15076,7 +15076,7 @@
         <v>117</v>
       </c>
       <c r="N304" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B304, $C$2:$C$620, C304, $D$2:$D$620, D304, $E$2:$E$620, E304) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -15122,7 +15122,7 @@
         <v>250</v>
       </c>
       <c r="N305" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B305, $C$2:$C$620, C305, $D$2:$D$620, D305, $E$2:$E$620, E305) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -15156,7 +15156,7 @@
       </c>
       <c r="J306" s="32"/>
       <c r="N306" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B306, $C$2:$C$620, C306, $D$2:$D$620, D306, $E$2:$E$620, E306) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -15192,7 +15192,7 @@
         <v>151</v>
       </c>
       <c r="N307" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B307, $C$2:$C$620, C307, $D$2:$D$620, D307, $E$2:$E$620, E307) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -15238,7 +15238,7 @@
         <v>250</v>
       </c>
       <c r="N308" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B308, $C$2:$C$620, C308, $D$2:$D$620, D308, $E$2:$E$620, E308) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
       <c r="P308" s="27"/>
@@ -15273,7 +15273,7 @@
       </c>
       <c r="J309" s="32"/>
       <c r="N309" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B309, $C$2:$C$620, C309, $D$2:$D$620, D309, $E$2:$E$620, E309) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -15309,7 +15309,7 @@
         <v>117</v>
       </c>
       <c r="N310" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B310, $C$2:$C$620, C310, $D$2:$D$620, D310, $E$2:$E$620, E310) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -15345,7 +15345,7 @@
         <v>116</v>
       </c>
       <c r="N311" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B311, $C$2:$C$620, C311, $D$2:$D$620, D311, $E$2:$E$620, E311) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -15379,7 +15379,7 @@
       </c>
       <c r="J312" s="32"/>
       <c r="N312" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B312, $C$2:$C$620, C312, $D$2:$D$620, D312, $E$2:$E$620, E312) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
       <c r="O312" s="27"/>
@@ -15414,7 +15414,7 @@
       </c>
       <c r="J313" s="32"/>
       <c r="N313" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B313, $C$2:$C$620, C313, $D$2:$D$620, D313, $E$2:$E$620, E313) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -15450,7 +15450,7 @@
         <v>54</v>
       </c>
       <c r="N314" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B314, $C$2:$C$620, C314, $D$2:$D$620, D314, $E$2:$E$620, E314) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -15484,7 +15484,7 @@
       </c>
       <c r="J315" s="32"/>
       <c r="N315" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B315, $C$2:$C$620, C315, $D$2:$D$620, D315, $E$2:$E$620, E315) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -15518,7 +15518,7 @@
       </c>
       <c r="J316" s="32"/>
       <c r="N316" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B316, $C$2:$C$620, C316, $D$2:$D$620, D316, $E$2:$E$620, E316) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -15564,7 +15564,7 @@
         <v>300</v>
       </c>
       <c r="N317" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B317, $C$2:$C$620, C317, $D$2:$D$620, D317, $E$2:$E$620, E317) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -15610,7 +15610,7 @@
         <v>235</v>
       </c>
       <c r="N318" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B318, $C$2:$C$620, C318, $D$2:$D$620, D318, $E$2:$E$620, E318) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -15656,7 +15656,7 @@
         <v>250</v>
       </c>
       <c r="N319" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B319, $C$2:$C$620, C319, $D$2:$D$620, D319, $E$2:$E$620, E319) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -15692,7 +15692,7 @@
         <v>117</v>
       </c>
       <c r="N320" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B320, $C$2:$C$620, C320, $D$2:$D$620, D320, $E$2:$E$620, E320) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -15728,7 +15728,7 @@
         <v>117</v>
       </c>
       <c r="N321" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B321, $C$2:$C$620, C321, $D$2:$D$620, D321, $E$2:$E$620, E321) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -15767,7 +15767,7 @@
       <c r="L322" s="25"/>
       <c r="M322" s="25"/>
       <c r="N322" s="27" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B322, $C$2:$C$620, C322, $D$2:$D$620, D322, $E$2:$E$620, E322) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
       <c r="O322" s="27"/>
@@ -15808,7 +15808,7 @@
       <c r="L323" s="25"/>
       <c r="M323" s="25"/>
       <c r="N323" s="27" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B323, $C$2:$C$620, C323, $D$2:$D$620, D323, $E$2:$E$620, E323) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
       <c r="O323" s="27"/>
@@ -15856,7 +15856,7 @@
         <v>250</v>
       </c>
       <c r="N324" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B324, $C$2:$C$620, C324, $D$2:$D$620, D324, $E$2:$E$620, E324) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>
@@ -15892,7 +15892,7 @@
         <v>116</v>
       </c>
       <c r="N325" s="10" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$620, B325, $C$2:$C$620, C325, $D$2:$D$620, D325, $E$2:$E$620, E325) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="12"/>
         <v>Unique</v>
       </c>
     </row>

</xml_diff>